<commit_message>
Add all current analysis files and interactive DMS heatmap
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/rna_analysis/I315RvI315X_significant_genes.xlsx
+++ b/results/rna_analysis/I315RvI315X_significant_genes.xlsx
@@ -393,22 +393,22 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>15.82244786348285</v>
+        <v>15.82244786348284</v>
       </c>
       <c r="B2">
-        <v>-3.818232755679578</v>
+        <v>-3.818432325716959</v>
       </c>
       <c r="C2">
-        <v>1.139268053631717</v>
+        <v>1.144281672202778</v>
       </c>
       <c r="D2">
-        <v>-3.351478823186479</v>
+        <v>-3.336968876173957</v>
       </c>
       <c r="E2">
-        <v>0.0008038118647128498</v>
+        <v>0.0008469743230532442</v>
       </c>
       <c r="F2">
-        <v>0.04030466554647633</v>
+        <v>0.04135178571995364</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -418,22 +418,22 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>78.33061449639634</v>
+        <v>78.33061449639632</v>
       </c>
       <c r="B3">
-        <v>-2.527748448503913</v>
+        <v>-2.52801082416236</v>
       </c>
       <c r="C3">
-        <v>0.555446472177581</v>
+        <v>0.5575902048313938</v>
       </c>
       <c r="D3">
-        <v>-4.550840765256981</v>
+        <v>-4.533814981428502</v>
       </c>
       <c r="E3">
-        <v>5.343197480849697E-06</v>
+        <v>5.792777544650812E-06</v>
       </c>
       <c r="F3">
-        <v>0.000712098239706574</v>
+        <v>0.0007500891340643065</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -443,22 +443,22 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>65.70749990864724</v>
+        <v>65.70749990864722</v>
       </c>
       <c r="B4">
-        <v>-2.085000602291968</v>
+        <v>-2.085009837101279</v>
       </c>
       <c r="C4">
-        <v>0.5265866120398852</v>
+        <v>0.5291411442741252</v>
       </c>
       <c r="D4">
-        <v>-3.959463751300316</v>
+        <v>-3.940366119065438</v>
       </c>
       <c r="E4">
-        <v>7.511824453383397E-05</v>
+        <v>8.13573459872741E-05</v>
       </c>
       <c r="F4">
-        <v>0.006505065410091361</v>
+        <v>0.006768113067578204</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -468,22 +468,22 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>358.4423446757558</v>
+        <v>358.4423446757557</v>
       </c>
       <c r="B5">
-        <v>-2.527544459977121</v>
+        <v>-2.527572163768402</v>
       </c>
       <c r="C5">
-        <v>0.2930839601282322</v>
+        <v>0.2937731014919495</v>
       </c>
       <c r="D5">
-        <v>-8.623960379378152</v>
+        <v>-8.603824349240726</v>
       </c>
       <c r="E5">
-        <v>6.467750448400369E-18</v>
+        <v>7.710294921412992E-18</v>
       </c>
       <c r="F5">
-        <v>8.933139323867891E-15</v>
+        <v>9.567833472896739E-15</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -496,19 +496,19 @@
         <v>21.2470271952201</v>
       </c>
       <c r="B6">
-        <v>-7.840551269502123</v>
+        <v>-7.840537748266037</v>
       </c>
       <c r="C6">
-        <v>1.702479042477425</v>
+        <v>1.705513434477037</v>
       </c>
       <c r="D6">
-        <v>-4.605373149317984</v>
+        <v>-4.597171496728894</v>
       </c>
       <c r="E6">
-        <v>4.1172690271905E-06</v>
+        <v>4.2826510215664E-06</v>
       </c>
       <c r="F6">
-        <v>0.0005792006326861598</v>
+        <v>0.0005850729941481216</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -518,22 +518,22 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>37.4725890905362</v>
+        <v>37.47258909053619</v>
       </c>
       <c r="B7">
-        <v>-2.560524566806978</v>
+        <v>-2.560793548738681</v>
       </c>
       <c r="C7">
-        <v>0.7755299533911167</v>
+        <v>0.7787831604107105</v>
       </c>
       <c r="D7">
-        <v>-3.30164496627205</v>
+        <v>-3.288198408640711</v>
       </c>
       <c r="E7">
-        <v>0.0009611965056134749</v>
+        <v>0.001008307521321671</v>
       </c>
       <c r="F7">
-        <v>0.04621347629678963</v>
+        <v>0.04721606069182704</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -543,22 +543,22 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>63.05175411558329</v>
+        <v>63.05175411558328</v>
       </c>
       <c r="B8">
-        <v>-2.060083846343292</v>
+        <v>-2.060215370232501</v>
       </c>
       <c r="C8">
-        <v>0.5968191937832021</v>
+        <v>0.5993759287986966</v>
       </c>
       <c r="D8">
-        <v>-3.451772107536522</v>
+        <v>-3.437267449765128</v>
       </c>
       <c r="E8">
-        <v>0.0005569178894509746</v>
+        <v>0.0005876150676422978</v>
       </c>
       <c r="F8">
-        <v>0.03032707345673354</v>
+        <v>0.0309193497253055</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -571,19 +571,19 @@
         <v>13.05570814905536</v>
       </c>
       <c r="B9">
-        <v>-4.747556550445832</v>
+        <v>-4.747872277620151</v>
       </c>
       <c r="C9">
-        <v>1.30705118022276</v>
+        <v>1.312577873218235</v>
       </c>
       <c r="D9">
-        <v>-3.632265225939133</v>
+        <v>-3.617211880906626</v>
       </c>
       <c r="E9">
-        <v>0.0002809441433080507</v>
+        <v>0.0002977935251682902</v>
       </c>
       <c r="F9">
-        <v>0.01863923305362103</v>
+        <v>0.01910781843741542</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -593,22 +593,22 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>66.68205138211145</v>
+        <v>66.68205138211144</v>
       </c>
       <c r="B10">
-        <v>-7.057305744375935</v>
+        <v>-7.057275377174677</v>
       </c>
       <c r="C10">
-        <v>1.143400989590188</v>
+        <v>1.144683613587754</v>
       </c>
       <c r="D10">
-        <v>-6.172205384311746</v>
+        <v>-6.165262866876579</v>
       </c>
       <c r="E10">
-        <v>6.734393869488176E-10</v>
+        <v>7.036614732492652E-10</v>
       </c>
       <c r="F10">
-        <v>2.623478104080355E-07</v>
+        <v>2.578597552449002E-07</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -621,19 +621,19 @@
         <v>10.4014849534835</v>
       </c>
       <c r="B11">
-        <v>-6.807213565539941</v>
+        <v>-6.80723329259883</v>
       </c>
       <c r="C11">
-        <v>1.990381539439422</v>
+        <v>1.995934495426051</v>
       </c>
       <c r="D11">
-        <v>-3.420054612974932</v>
+        <v>-3.410549448490675</v>
       </c>
       <c r="E11">
-        <v>0.0006260856516422702</v>
+        <v>0.0006483212686252391</v>
       </c>
       <c r="F11">
-        <v>0.0330281920326424</v>
+        <v>0.03317578010686748</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -643,22 +643,22 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>11.58904434141501</v>
+        <v>11.589044341415</v>
       </c>
       <c r="B12">
-        <v>-6.965321457694807</v>
+        <v>-6.965316463680563</v>
       </c>
       <c r="C12">
-        <v>1.87835448512763</v>
+        <v>1.883467344265228</v>
       </c>
       <c r="D12">
-        <v>-3.708203916164167</v>
+        <v>-3.69813497690232</v>
       </c>
       <c r="E12">
-        <v>0.0002087345388834404</v>
+        <v>0.0002171893954764026</v>
       </c>
       <c r="F12">
-        <v>0.01438071635003349</v>
+        <v>0.01463424112234892</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -668,22 +668,22 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>200.908487972208</v>
+        <v>200.9084879722079</v>
       </c>
       <c r="B13">
-        <v>-2.622469954253549</v>
+        <v>-2.622491916304765</v>
       </c>
       <c r="C13">
-        <v>0.3475323234138423</v>
+        <v>0.3486801213727422</v>
       </c>
       <c r="D13">
-        <v>-7.545974223326288</v>
+        <v>-7.521197096009088</v>
       </c>
       <c r="E13">
-        <v>4.489188421040597E-14</v>
+        <v>5.427695288075022E-14</v>
       </c>
       <c r="F13">
-        <v>4.262764980054361E-11</v>
+        <v>4.754341796160303E-11</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -693,22 +693,22 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>283.1645770248061</v>
+        <v>283.164577024806</v>
       </c>
       <c r="B14">
-        <v>-2.01023529890834</v>
+        <v>-2.010226103845255</v>
       </c>
       <c r="C14">
-        <v>0.3138494371124229</v>
+        <v>0.3147134319698001</v>
       </c>
       <c r="D14">
-        <v>-6.405094485443544</v>
+        <v>-6.387481116592941</v>
       </c>
       <c r="E14">
-        <v>1.502762872447744E-10</v>
+        <v>1.686404251136791E-10</v>
       </c>
       <c r="F14">
-        <v>6.523278948885305E-08</v>
+        <v>6.975623806577212E-08</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -718,22 +718,22 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>60.32164293018688</v>
+        <v>60.32164293018687</v>
       </c>
       <c r="B15">
-        <v>-3.215731509658428</v>
+        <v>-3.215995527294079</v>
       </c>
       <c r="C15">
-        <v>0.7194055824470437</v>
+        <v>0.7224118633243894</v>
       </c>
       <c r="D15">
-        <v>-4.469984092589582</v>
+        <v>-4.451747944025636</v>
       </c>
       <c r="E15">
-        <v>7.822541499080078E-06</v>
+        <v>8.517410999623019E-06</v>
       </c>
       <c r="F15">
-        <v>0.0009903989416293636</v>
+        <v>0.001039874426860547</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -743,22 +743,22 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>39.94942595346182</v>
+        <v>39.94942595346181</v>
       </c>
       <c r="B16">
-        <v>-4.162345159229525</v>
+        <v>-4.163996323425295</v>
       </c>
       <c r="C16">
-        <v>0.8713554985419515</v>
+        <v>0.8753650169516645</v>
       </c>
       <c r="D16">
-        <v>-4.776862217768088</v>
+        <v>-4.756868555160939</v>
       </c>
       <c r="E16">
-        <v>1.780516825502956E-06</v>
+        <v>1.966191028259618E-06</v>
       </c>
       <c r="F16">
-        <v>0.0002788803312357362</v>
+        <v>0.0002957429353718584</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -771,19 +771,19 @@
         <v>81.84227223514216</v>
       </c>
       <c r="B17">
-        <v>-4.557595209851749</v>
+        <v>-4.557812822246598</v>
       </c>
       <c r="C17">
-        <v>0.6212661961712153</v>
+        <v>0.6233024488649926</v>
       </c>
       <c r="D17">
-        <v>-7.335978100755571</v>
+        <v>-7.312361487663305</v>
       </c>
       <c r="E17">
-        <v>2.201080125622712E-13</v>
+        <v>2.624878048364913E-13</v>
       </c>
       <c r="F17">
-        <v>1.672050517429293E-10</v>
+        <v>1.77668450082736E-10</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -793,22 +793,22 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>11.59692815699415</v>
+        <v>11.59692815699414</v>
       </c>
       <c r="B18">
-        <v>-6.966168386418725</v>
+        <v>-6.96616509234273</v>
       </c>
       <c r="C18">
-        <v>1.876858738835419</v>
+        <v>1.881969964502211</v>
       </c>
       <c r="D18">
-        <v>-3.711610385095469</v>
+        <v>-3.701528304775741</v>
       </c>
       <c r="E18">
-        <v>0.0002059448200475793</v>
+        <v>0.0002143047441297483</v>
       </c>
       <c r="F18">
-        <v>0.01428730434238755</v>
+        <v>0.0145717440403474</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -818,22 +818,22 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>74.3693274599943</v>
+        <v>74.36932745999428</v>
       </c>
       <c r="B19">
-        <v>-2.101416599999369</v>
+        <v>-2.10134571218527</v>
       </c>
       <c r="C19">
-        <v>0.5156114362235724</v>
+        <v>0.5179329142014588</v>
       </c>
       <c r="D19">
-        <v>-4.075581828422017</v>
+        <v>-4.05717739608245</v>
       </c>
       <c r="E19">
-        <v>4.589943791745028E-05</v>
+        <v>4.966935542509901E-05</v>
       </c>
       <c r="F19">
-        <v>0.004441720766113516</v>
+        <v>0.004651738186384587</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -846,19 +846,19 @@
         <v>21.22360653388426</v>
       </c>
       <c r="B20">
-        <v>-6.203568168156697</v>
+        <v>-6.205071987246882</v>
       </c>
       <c r="C20">
-        <v>1.716552569569615</v>
+        <v>1.720423093291089</v>
       </c>
       <c r="D20">
-        <v>-3.613969230031851</v>
+        <v>-3.606712797243886</v>
       </c>
       <c r="E20">
-        <v>0.0003015448641933453</v>
+        <v>0.0003101005628377596</v>
       </c>
       <c r="F20">
-        <v>0.01949519626250849</v>
+        <v>0.01954902499324052</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -871,19 +871,19 @@
         <v>59.4084766306208</v>
       </c>
       <c r="B21">
-        <v>-2.234629558600185</v>
+        <v>-2.234601310358754</v>
       </c>
       <c r="C21">
-        <v>0.5763062719215903</v>
+        <v>0.5789262452523449</v>
       </c>
       <c r="D21">
-        <v>-3.877503451678935</v>
+        <v>-3.859906730234222</v>
       </c>
       <c r="E21">
-        <v>0.0001055338308374151</v>
+        <v>0.0001134303115310421</v>
       </c>
       <c r="F21">
-        <v>0.008483468211179086</v>
+        <v>0.008889951415835519</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -893,22 +893,22 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>96.362100491175</v>
+        <v>96.36210049117497</v>
       </c>
       <c r="B22">
-        <v>-3.863207743383831</v>
+        <v>-3.86317723740627</v>
       </c>
       <c r="C22">
-        <v>0.5017999273942204</v>
+        <v>0.5036301513645767</v>
       </c>
       <c r="D22">
-        <v>-7.698701280099718</v>
+        <v>-7.67066313829516</v>
       </c>
       <c r="E22">
-        <v>1.374560836958903E-14</v>
+        <v>1.711093841328585E-14</v>
       </c>
       <c r="F22">
-        <v>1.491693056851187E-11</v>
+        <v>1.592493649451498E-11</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -921,19 +921,19 @@
         <v>241.5269198680776</v>
       </c>
       <c r="B23">
-        <v>-2.280345352013371</v>
+        <v>-2.280356852343163</v>
       </c>
       <c r="C23">
-        <v>0.3138483107074974</v>
+        <v>0.3148588576557497</v>
       </c>
       <c r="D23">
-        <v>-7.265756335832643</v>
+        <v>-7.242473244428736</v>
       </c>
       <c r="E23">
-        <v>3.709567454338623E-13</v>
+        <v>4.4057537465687E-13</v>
       </c>
       <c r="F23">
-        <v>2.4504112319029E-10</v>
+        <v>2.733586626673105E-10</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -943,22 +943,22 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>24.91992331147513</v>
+        <v>24.91992331147515</v>
       </c>
       <c r="B24">
-        <v>4.138091589558424</v>
+        <v>4.13904301389862</v>
       </c>
       <c r="C24">
-        <v>1.082871589259292</v>
+        <v>1.086596189935687</v>
       </c>
       <c r="D24">
-        <v>3.821405631658478</v>
+        <v>3.809182336764498</v>
       </c>
       <c r="E24">
-        <v>0.0001326931897576785</v>
+        <v>0.00013942711200239</v>
       </c>
       <c r="F24">
-        <v>0.01013069161803221</v>
+        <v>0.01038104562413795</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -971,19 +971,19 @@
         <v>1734.972591843603</v>
       </c>
       <c r="B25">
-        <v>2.288180450654952</v>
+        <v>2.288179443360047</v>
       </c>
       <c r="C25">
-        <v>0.2085228505590656</v>
+        <v>0.2084104684804206</v>
       </c>
       <c r="D25">
-        <v>10.97328395674702</v>
+        <v>10.97919629490691</v>
       </c>
       <c r="E25">
-        <v>5.137200393894983E-28</v>
+        <v>4.811856423195965E-28</v>
       </c>
       <c r="F25">
-        <v>1.951237139611162E-24</v>
+        <v>1.791333849945278E-24</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -993,22 +993,22 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>29.63363271061307</v>
+        <v>29.63363271061306</v>
       </c>
       <c r="B26">
-        <v>4.879397701132997</v>
+        <v>4.877366366846363</v>
       </c>
       <c r="C26">
-        <v>1.274301314867839</v>
+        <v>1.277567943411351</v>
       </c>
       <c r="D26">
-        <v>3.829076878602335</v>
+        <v>3.817696265783613</v>
       </c>
       <c r="E26">
-        <v>0.0001286248247562089</v>
+        <v>0.0001347036183529965</v>
       </c>
       <c r="F26">
-        <v>0.009952758377774021</v>
+        <v>0.01013066454997208</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1021,19 +1021,19 @@
         <v>108.0612150378456</v>
       </c>
       <c r="B27">
-        <v>2.629790893781912</v>
+        <v>2.629647201030882</v>
       </c>
       <c r="C27">
-        <v>0.4669301037271905</v>
+        <v>0.4687834870821028</v>
       </c>
       <c r="D27">
-        <v>5.632086842955832</v>
+        <v>5.609513290237388</v>
       </c>
       <c r="E27">
-        <v>1.780419854688578E-08</v>
+        <v>2.028964164462644E-08</v>
       </c>
       <c r="F27">
-        <v>4.755407473949403E-06</v>
+        <v>5.209190581554005E-06</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1043,22 +1043,22 @@
     </row>
     <row r="28">
       <c r="A28">
-        <v>36.47614641937907</v>
+        <v>36.47614641937909</v>
       </c>
       <c r="B28">
-        <v>4.415046634901842</v>
+        <v>4.415194029521548</v>
       </c>
       <c r="C28">
-        <v>0.7973092622340416</v>
+        <v>0.8005110411356119</v>
       </c>
       <c r="D28">
-        <v>5.537433018815041</v>
+        <v>5.515469247317458</v>
       </c>
       <c r="E28">
-        <v>3.069370196414248E-08</v>
+        <v>3.478505691647237E-08</v>
       </c>
       <c r="F28">
-        <v>7.644744490839618E-06</v>
+        <v>8.354585202309518E-06</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1068,22 +1068,22 @@
     </row>
     <row r="29">
       <c r="A29">
-        <v>309.5406636768796</v>
+        <v>309.5406636768797</v>
       </c>
       <c r="B29">
-        <v>4.661976251554973</v>
+        <v>4.66197992540449</v>
       </c>
       <c r="C29">
-        <v>0.3427378148632071</v>
+        <v>0.3434281406109266</v>
       </c>
       <c r="D29">
-        <v>13.60216483090917</v>
+        <v>13.57483378360103</v>
       </c>
       <c r="E29">
-        <v>3.887537223599322E-42</v>
+        <v>5.647166354263744E-42</v>
       </c>
       <c r="F29">
-        <v>5.906335303814449E-38</v>
+        <v>8.40919541813414E-38</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1093,22 +1093,22 @@
     </row>
     <row r="30">
       <c r="A30">
-        <v>463.6679944099959</v>
+        <v>463.667994409996</v>
       </c>
       <c r="B30">
-        <v>3.398855174498036</v>
+        <v>3.398871841887403</v>
       </c>
       <c r="C30">
-        <v>0.2921718662701005</v>
+        <v>0.2926832167519232</v>
       </c>
       <c r="D30">
-        <v>11.63306795376369</v>
+        <v>11.6128006231675</v>
       </c>
       <c r="E30">
-        <v>2.798551981791887E-31</v>
+        <v>3.548009753455893E-31</v>
       </c>
       <c r="F30">
-        <v>1.421579208015857E-27</v>
+        <v>1.761113774623724E-27</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1121,19 +1121,19 @@
         <v>52.59310021442771</v>
       </c>
       <c r="B31">
-        <v>5.370641195664951</v>
+        <v>5.368027176215598</v>
       </c>
       <c r="C31">
-        <v>0.9682950844236587</v>
+        <v>0.9706075158265272</v>
       </c>
       <c r="D31">
-        <v>5.546492264660853</v>
+        <v>5.530584802492921</v>
       </c>
       <c r="E31">
-        <v>2.914575157633951E-08</v>
+        <v>3.191649548284495E-08</v>
       </c>
       <c r="F31">
-        <v>7.380190061655435E-06</v>
+        <v>7.791287446476134E-06</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1146,19 +1146,19 @@
         <v>14.28691612518962</v>
       </c>
       <c r="B32">
-        <v>7.29004562437766</v>
+        <v>7.290066344571058</v>
       </c>
       <c r="C32">
-        <v>1.806557544794852</v>
+        <v>1.810850411686486</v>
       </c>
       <c r="D32">
-        <v>4.03532433571359</v>
+        <v>4.02576949345123</v>
       </c>
       <c r="E32">
-        <v>5.452692253188939E-05</v>
+        <v>5.678929894658269E-05</v>
       </c>
       <c r="F32">
-        <v>0.005113750210043182</v>
+        <v>0.005188033439347011</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1171,19 +1171,19 @@
         <v>24.86873791295172</v>
       </c>
       <c r="B33">
-        <v>3.707129046088363</v>
+        <v>3.706345564422659</v>
       </c>
       <c r="C33">
-        <v>1.000863833814558</v>
+        <v>1.004808998772144</v>
       </c>
       <c r="D33">
-        <v>3.703929466568404</v>
+        <v>3.688607057611681</v>
       </c>
       <c r="E33">
-        <v>0.0002122853064832279</v>
+        <v>0.0002254851457343134</v>
       </c>
       <c r="F33">
-        <v>0.014528156132431</v>
+        <v>0.01498972904075742</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1196,19 +1196,19 @@
         <v>327.2001623700594</v>
       </c>
       <c r="B34">
-        <v>2.152885851763551</v>
+        <v>2.152888964094629</v>
       </c>
       <c r="C34">
-        <v>0.2942308769262089</v>
+        <v>0.2949887716594909</v>
       </c>
       <c r="D34">
-        <v>7.316994987930786</v>
+        <v>7.298206477430725</v>
       </c>
       <c r="E34">
-        <v>2.535853198520343E-13</v>
+        <v>2.916288747762528E-13</v>
       </c>
       <c r="F34">
-        <v>1.767702616480132E-10</v>
+        <v>1.888106771431818E-10</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1218,22 +1218,22 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>57.61185103135259</v>
+        <v>57.6118510313526</v>
       </c>
       <c r="B35">
-        <v>3.564675243958033</v>
+        <v>3.564680144335354</v>
       </c>
       <c r="C35">
-        <v>0.6329626410887609</v>
+        <v>0.6354501547952686</v>
       </c>
       <c r="D35">
-        <v>5.631730867759312</v>
+        <v>5.609692778316868</v>
       </c>
       <c r="E35">
-        <v>1.78409942746736E-08</v>
+        <v>2.026861048896341E-08</v>
       </c>
       <c r="F35">
-        <v>4.755407473949403E-06</v>
+        <v>5.209190581554005E-06</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1243,22 +1243,22 @@
     </row>
     <row r="36">
       <c r="A36">
-        <v>122.0344844727188</v>
+        <v>122.0344844727189</v>
       </c>
       <c r="B36">
-        <v>2.389128313446546</v>
+        <v>2.389128100524367</v>
       </c>
       <c r="C36">
-        <v>0.4407106698912049</v>
+        <v>0.4423734514305371</v>
       </c>
       <c r="D36">
-        <v>5.421081168822922</v>
+        <v>5.400704072087643</v>
       </c>
       <c r="E36">
-        <v>5.923965250004834E-08</v>
+        <v>6.63798502290756E-08</v>
       </c>
       <c r="F36">
-        <v>1.323570647695933E-05</v>
+        <v>1.432554130088645E-05</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1271,19 +1271,19 @@
         <v>121.595790741968</v>
       </c>
       <c r="B37">
-        <v>3.158782804333514</v>
+        <v>3.158771851394899</v>
       </c>
       <c r="C37">
-        <v>0.4351009371681372</v>
+        <v>0.4367247509869076</v>
       </c>
       <c r="D37">
-        <v>7.259885085268977</v>
+        <v>7.232866569290448</v>
       </c>
       <c r="E37">
-        <v>3.874193168784756E-13</v>
+        <v>4.729039875606714E-13</v>
       </c>
       <c r="F37">
-        <v>2.452525700556116E-10</v>
+        <v>2.816805311506383E-10</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1296,19 +1296,19 @@
         <v>25.13439720292818</v>
       </c>
       <c r="B38">
-        <v>4.577934309927784</v>
+        <v>4.577703565949886</v>
       </c>
       <c r="C38">
-        <v>1.117706316688388</v>
+        <v>1.121892845238772</v>
       </c>
       <c r="D38">
-        <v>4.095829326161082</v>
+        <v>4.080339388362543</v>
       </c>
       <c r="E38">
-        <v>4.206597651757658E-05</v>
+        <v>4.49699930388974E-05</v>
       </c>
       <c r="F38">
-        <v>0.004123279878913167</v>
+        <v>0.004292616450911674</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1321,19 +1321,19 @@
         <v>115.9057335674553</v>
       </c>
       <c r="B39">
-        <v>4.561034586632001</v>
+        <v>4.561023736215371</v>
       </c>
       <c r="C39">
-        <v>0.5350054653022167</v>
+        <v>0.5365938685761102</v>
       </c>
       <c r="D39">
-        <v>8.525211203320213</v>
+        <v>8.49995500007924</v>
       </c>
       <c r="E39">
-        <v>1.525312458028938E-17</v>
+        <v>1.896642064931846E-17</v>
       </c>
       <c r="F39">
-        <v>1.782620936525665E-14</v>
+        <v>2.017349784921437E-14</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1346,19 +1346,19 @@
         <v>84.61421682235719</v>
       </c>
       <c r="B40">
-        <v>2.586162904635926</v>
+        <v>2.586049324884496</v>
       </c>
       <c r="C40">
-        <v>0.5345132102837121</v>
+        <v>0.5365231613677195</v>
       </c>
       <c r="D40">
-        <v>4.838351709330491</v>
+        <v>4.820014327605296</v>
       </c>
       <c r="E40">
-        <v>1.3092032038925E-06</v>
+        <v>1.435479116636061E-06</v>
       </c>
       <c r="F40">
-        <v>0.0002093760450183027</v>
+        <v>0.000222663745060704</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1368,22 +1368,22 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>3552.192452666699</v>
+        <v>3552.1924526667</v>
       </c>
       <c r="B41">
-        <v>2.399801487979943</v>
+        <v>2.399801271291311</v>
       </c>
       <c r="C41">
-        <v>0.2677664761343931</v>
+        <v>0.2675139396173747</v>
       </c>
       <c r="D41">
-        <v>8.962292526774235</v>
+        <v>8.970752233411639</v>
       </c>
       <c r="E41">
-        <v>3.179969183595624E-19</v>
+        <v>2.944962286207995E-19</v>
       </c>
       <c r="F41">
-        <v>5.368141311818701E-16</v>
+        <v>4.872603711547028E-16</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1393,22 +1393,22 @@
     </row>
     <row r="42">
       <c r="A42">
-        <v>45.35384803244658</v>
+        <v>45.35384803244659</v>
       </c>
       <c r="B42">
-        <v>2.393969180846306</v>
+        <v>2.393633684557955</v>
       </c>
       <c r="C42">
-        <v>0.6690678205989549</v>
+        <v>0.6721570282000628</v>
       </c>
       <c r="D42">
-        <v>3.578066538461237</v>
+        <v>3.561122749795167</v>
       </c>
       <c r="E42">
-        <v>0.0003461453419212335</v>
+        <v>0.0003692723874481051</v>
       </c>
       <c r="F42">
-        <v>0.02155322204839877</v>
+        <v>0.02238762914404021</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1421,19 +1421,19 @@
         <v>151.2196261945458</v>
       </c>
       <c r="B43">
-        <v>2.409113801270647</v>
+        <v>2.409080433237952</v>
       </c>
       <c r="C43">
-        <v>0.4030514931232236</v>
+        <v>0.4044686183623951</v>
       </c>
       <c r="D43">
-        <v>5.977186147116236</v>
+        <v>5.95616155090546</v>
       </c>
       <c r="E43">
-        <v>2.270247380969633E-09</v>
+        <v>2.58231074788386E-09</v>
       </c>
       <c r="F43">
-        <v>7.664859657571474E-07</v>
+        <v>8.359388988421425E-07</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1443,22 +1443,22 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>87.18600709829724</v>
+        <v>87.18600709829725</v>
       </c>
       <c r="B44">
-        <v>2.434649427184934</v>
+        <v>2.434386449489563</v>
       </c>
       <c r="C44">
-        <v>0.4903443082344558</v>
+        <v>0.492451100057347</v>
       </c>
       <c r="D44">
-        <v>4.965183415610931</v>
+        <v>4.943407475800285</v>
       </c>
       <c r="E44">
-        <v>6.863617169753448E-07</v>
+        <v>7.676879271952801E-07</v>
       </c>
       <c r="F44">
-        <v>0.0001198608455862806</v>
+        <v>0.000129905010498465</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1468,22 +1468,22 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>31.5155312027357</v>
+        <v>31.51553120273572</v>
       </c>
       <c r="B45">
-        <v>3.442894468941805</v>
+        <v>3.443168217026635</v>
       </c>
       <c r="C45">
-        <v>0.8623443238295615</v>
+        <v>0.8658511349057363</v>
       </c>
       <c r="D45">
-        <v>3.992482322667063</v>
+        <v>3.976628404375179</v>
       </c>
       <c r="E45">
-        <v>6.538520864940564E-05</v>
+        <v>6.989926281508013E-05</v>
       </c>
       <c r="F45">
-        <v>0.005913080208395357</v>
+        <v>0.006086958611575194</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1493,22 +1493,22 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>44.94799521693492</v>
+        <v>44.94799521693493</v>
       </c>
       <c r="B46">
-        <v>2.141226069412558</v>
+        <v>2.141229285154364</v>
       </c>
       <c r="C46">
-        <v>0.6409782106712743</v>
+        <v>0.6440838320530912</v>
       </c>
       <c r="D46">
-        <v>3.340559840825363</v>
+        <v>3.32445743643176</v>
       </c>
       <c r="E46">
-        <v>0.0008360966044834527</v>
+        <v>0.0008859075519591485</v>
       </c>
       <c r="F46">
-        <v>0.04164099573821623</v>
+        <v>0.04283132907864832</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1518,22 +1518,22 @@
     </row>
     <row r="47">
       <c r="A47">
-        <v>64.60978180309225</v>
+        <v>64.60978180309226</v>
       </c>
       <c r="B47">
-        <v>2.554827070349844</v>
+        <v>2.553327702235356</v>
       </c>
       <c r="C47">
-        <v>0.6792811885335588</v>
+        <v>0.6818122939768249</v>
       </c>
       <c r="D47">
-        <v>3.761074373140287</v>
+        <v>3.744912969143594</v>
       </c>
       <c r="E47">
-        <v>0.0001691851122088497</v>
+        <v>0.0001804563201681291</v>
       </c>
       <c r="F47">
-        <v>0.01238253081756086</v>
+        <v>0.01285729695513689</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>94.25949285756298</v>
+        <v>94.25949285756299</v>
       </c>
       <c r="B48">
-        <v>2.032249763135095</v>
+        <v>2.032230119457117</v>
       </c>
       <c r="C48">
-        <v>0.4705691076089522</v>
+        <v>0.4725465544862356</v>
       </c>
       <c r="D48">
-        <v>4.318706286227178</v>
+        <v>4.300592397010721</v>
       </c>
       <c r="E48">
-        <v>1.569464843843592E-05</v>
+        <v>1.7034212774862E-05</v>
       </c>
       <c r="F48">
-        <v>0.001806430255493613</v>
+        <v>0.001892958674854254</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1568,22 +1568,22 @@
     </row>
     <row r="49">
       <c r="A49">
-        <v>849.0613273156116</v>
+        <v>849.0613273156119</v>
       </c>
       <c r="B49">
-        <v>2.543136991827881</v>
+        <v>2.543121322469782</v>
       </c>
       <c r="C49">
-        <v>0.2780572088805795</v>
+        <v>0.2782117277782426</v>
       </c>
       <c r="D49">
-        <v>9.146092640669899</v>
+        <v>9.140956575694236</v>
       </c>
       <c r="E49">
-        <v>5.903006845693231E-20</v>
+        <v>6.190232277845077E-20</v>
       </c>
       <c r="F49">
-        <v>1.121054787582716E-16</v>
+        <v>1.152234360617388E-16</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -1593,22 +1593,22 @@
     </row>
     <row r="50">
       <c r="A50">
-        <v>36.10880364036268</v>
+        <v>36.10880364036269</v>
       </c>
       <c r="B50">
-        <v>4.096140593825356</v>
+        <v>4.096562631476697</v>
       </c>
       <c r="C50">
-        <v>0.8988673717668629</v>
+        <v>0.9019441802489455</v>
       </c>
       <c r="D50">
-        <v>4.557002203532828</v>
+        <v>4.541924790008629</v>
       </c>
       <c r="E50">
-        <v>5.188887997080506E-06</v>
+        <v>5.574292927553776E-06</v>
       </c>
       <c r="F50">
-        <v>0.0007045958097028106</v>
+        <v>0.0007345734157894096</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -1621,19 +1621,19 @@
         <v>53.36236045804426</v>
       </c>
       <c r="B51">
-        <v>2.190589940032881</v>
+        <v>2.190549629578005</v>
       </c>
       <c r="C51">
-        <v>0.6192518200010759</v>
+        <v>0.6220073455568124</v>
       </c>
       <c r="D51">
-        <v>3.537478404228307</v>
+        <v>3.521742380095295</v>
       </c>
       <c r="E51">
-        <v>0.0004039672201256894</v>
+        <v>0.0004287205494252015</v>
       </c>
       <c r="F51">
-        <v>0.02444412718393009</v>
+        <v>0.02464894865440415</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1643,22 +1643,22 @@
     </row>
     <row r="52">
       <c r="A52">
-        <v>212.8733222309916</v>
+        <v>212.8733222309917</v>
       </c>
       <c r="B52">
-        <v>2.333176361812052</v>
+        <v>2.333184554562516</v>
       </c>
       <c r="C52">
-        <v>0.3291909572686729</v>
+        <v>0.3303100644157576</v>
       </c>
       <c r="D52">
-        <v>7.087607694848688</v>
+        <v>7.063619325948734</v>
       </c>
       <c r="E52">
-        <v>1.364501124702795E-12</v>
+        <v>1.622207708126772E-12</v>
       </c>
       <c r="F52">
-        <v>7.403880567003414E-10</v>
+        <v>8.329756890246816E-10</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -1671,19 +1671,19 @@
         <v>40.40895379628694</v>
       </c>
       <c r="B53">
-        <v>3.017043577690328</v>
+        <v>3.01710735983772</v>
       </c>
       <c r="C53">
-        <v>0.7365778586649325</v>
+        <v>0.7396952527169344</v>
       </c>
       <c r="D53">
-        <v>4.096028060304177</v>
+        <v>4.078851863325805</v>
       </c>
       <c r="E53">
-        <v>4.202990094452793E-05</v>
+        <v>4.525866302010767E-05</v>
       </c>
       <c r="F53">
-        <v>0.004123279878913167</v>
+        <v>0.00429265446517467</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -1696,19 +1696,19 @@
         <v>49.53375117078028</v>
       </c>
       <c r="B54">
-        <v>2.756694557892928</v>
+        <v>2.756657120120685</v>
       </c>
       <c r="C54">
-        <v>0.6547619016855338</v>
+        <v>0.6576606159873766</v>
       </c>
       <c r="D54">
-        <v>4.210224435472578</v>
+        <v>4.191610464588924</v>
       </c>
       <c r="E54">
-        <v>2.551171246313579E-05</v>
+        <v>2.769812689947202E-05</v>
       </c>
       <c r="F54">
-        <v>0.002748932251435617</v>
+        <v>0.002884285368252013</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -1721,19 +1721,19 @@
         <v>147.9692373485587</v>
       </c>
       <c r="B55">
-        <v>4.938809132262872</v>
+        <v>5.079019104408325</v>
       </c>
       <c r="C55">
-        <v>1.258851941380601</v>
+        <v>0.5771803291079789</v>
       </c>
       <c r="D55">
-        <v>3.923264499911253</v>
+        <v>8.799709290609144</v>
       </c>
       <c r="E55">
-        <v>8.735715387618356E-05</v>
+        <v>1.371710262717534E-18</v>
       </c>
       <c r="F55">
-        <v>0.0072525532177096</v>
+        <v>2.04261375221268E-15</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -1743,22 +1743,22 @@
     </row>
     <row r="56">
       <c r="A56">
-        <v>719.4771374075194</v>
+        <v>719.4771374075196</v>
       </c>
       <c r="B56">
-        <v>2.286200056443219</v>
+        <v>2.286201946680802</v>
       </c>
       <c r="C56">
-        <v>0.2315685555192145</v>
+        <v>0.2318098964209964</v>
       </c>
       <c r="D56">
-        <v>9.872670541633708</v>
+        <v>9.862400104475123</v>
       </c>
       <c r="E56">
-        <v>5.468884710196201E-23</v>
+        <v>6.05835964983191E-23</v>
       </c>
       <c r="F56">
-        <v>1.384812756700181E-19</v>
+        <v>1.50358389242745E-19</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -1771,19 +1771,19 @@
         <v>22.10531726000153</v>
       </c>
       <c r="B57">
-        <v>3.598600276767161</v>
+        <v>3.598487583579796</v>
       </c>
       <c r="C57">
-        <v>1.015111722146831</v>
+        <v>1.019385487299151</v>
       </c>
       <c r="D57">
-        <v>3.545028786739437</v>
+        <v>3.530055733002382</v>
       </c>
       <c r="E57">
-        <v>0.0003925702100076098</v>
+        <v>0.0004154721363974793</v>
       </c>
       <c r="F57">
-        <v>0.02385727680258246</v>
+        <v>0.02442228210589323</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -1793,22 +1793,22 @@
     </row>
     <row r="58">
       <c r="A58">
-        <v>38.49018163226332</v>
+        <v>38.49018163226334</v>
       </c>
       <c r="B58">
-        <v>3.555288662891464</v>
+        <v>3.55543821266515</v>
       </c>
       <c r="C58">
-        <v>0.7804612663396689</v>
+        <v>0.7835496481184971</v>
       </c>
       <c r="D58">
-        <v>4.555368493257353</v>
+        <v>4.537604249076834</v>
       </c>
       <c r="E58">
-        <v>5.229382353184005E-06</v>
+        <v>5.689690592687107E-06</v>
       </c>
       <c r="F58">
-        <v>0.0007045958097028106</v>
+        <v>0.0007432033562781027</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -1821,19 +1821,19 @@
         <v>114.5195889976151</v>
       </c>
       <c r="B59">
-        <v>2.181184774461956</v>
+        <v>2.180156019343687</v>
       </c>
       <c r="C59">
-        <v>0.5477223767149414</v>
+        <v>0.5494467336177983</v>
       </c>
       <c r="D59">
-        <v>3.982281657988825</v>
+        <v>3.967911511619304</v>
       </c>
       <c r="E59">
-        <v>6.82568214862197E-05</v>
+        <v>7.250524396520857E-05</v>
       </c>
       <c r="F59">
-        <v>0.006014536664947958</v>
+        <v>0.006205032114286901</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -1846,19 +1846,19 @@
         <v>62.69406171744509</v>
       </c>
       <c r="B60">
-        <v>2.784032651565977</v>
+        <v>2.782819599842546</v>
       </c>
       <c r="C60">
-        <v>0.7403549900424523</v>
+        <v>0.7428997213096237</v>
       </c>
       <c r="D60">
-        <v>3.7604023596928</v>
+        <v>3.745888603830462</v>
       </c>
       <c r="E60">
-        <v>0.0001696402799417677</v>
+        <v>0.0001797563490058586</v>
       </c>
       <c r="F60">
-        <v>0.01238253081756086</v>
+        <v>0.01285729695513689</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -1868,22 +1868,22 @@
     </row>
     <row r="61">
       <c r="A61">
-        <v>26.8499561145288</v>
+        <v>26.84995611452881</v>
       </c>
       <c r="B61">
-        <v>4.344013807797931</v>
+        <v>4.344016184775032</v>
       </c>
       <c r="C61">
-        <v>1.003536611656235</v>
+        <v>1.007019891624974</v>
       </c>
       <c r="D61">
-        <v>4.328704859734594</v>
+        <v>4.313734237925852</v>
       </c>
       <c r="E61">
-        <v>1.499887756433281E-05</v>
+        <v>1.605198946335747E-05</v>
       </c>
       <c r="F61">
-        <v>0.001739526311716858</v>
+        <v>0.001810834659839818</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -1896,19 +1896,19 @@
         <v>40.25349730602554</v>
       </c>
       <c r="B62">
-        <v>2.202709530943947</v>
+        <v>2.202721601031583</v>
       </c>
       <c r="C62">
-        <v>0.6701878252499901</v>
+        <v>0.6735085568244885</v>
       </c>
       <c r="D62">
-        <v>3.286704783278185</v>
+        <v>3.270517618094044</v>
       </c>
       <c r="E62">
-        <v>0.00101367040662973</v>
+        <v>0.001073508550516887</v>
       </c>
       <c r="F62">
-        <v>0.04806715940000141</v>
+        <v>0.04940441735379195</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -1918,22 +1918,22 @@
     </row>
     <row r="63">
       <c r="A63">
-        <v>607.696170891666</v>
+        <v>607.6961708916663</v>
       </c>
       <c r="B63">
-        <v>2.50400671511725</v>
+        <v>2.504009690945951</v>
       </c>
       <c r="C63">
-        <v>0.2880363420910937</v>
+        <v>0.2883470764287143</v>
       </c>
       <c r="D63">
-        <v>8.693370763350892</v>
+        <v>8.68401275975828</v>
       </c>
       <c r="E63">
-        <v>3.518418380421245E-18</v>
+        <v>3.820459097352648E-18</v>
       </c>
       <c r="F63">
-        <v>5.345533045373997E-15</v>
+        <v>5.171859674425299E-15</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -1946,19 +1946,19 @@
         <v>40.94900172543174</v>
       </c>
       <c r="B64">
-        <v>2.889435997047413</v>
+        <v>2.889475216744197</v>
       </c>
       <c r="C64">
-        <v>0.7190286007607428</v>
+        <v>0.7221287872597971</v>
       </c>
       <c r="D64">
-        <v>4.01852721016987</v>
+        <v>4.001329496513567</v>
       </c>
       <c r="E64">
-        <v>5.856304715785029E-05</v>
+        <v>6.298757467077882E-05</v>
       </c>
       <c r="F64">
-        <v>0.005392414396783148</v>
+        <v>0.005607306677914486</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -1968,22 +1968,22 @@
     </row>
     <row r="65">
       <c r="A65">
-        <v>242.5754866664867</v>
+        <v>242.5754866664868</v>
       </c>
       <c r="B65">
-        <v>2.195381552126663</v>
+        <v>2.195365275161997</v>
       </c>
       <c r="C65">
-        <v>0.3415290547243144</v>
+        <v>0.3425378331671234</v>
       </c>
       <c r="D65">
-        <v>6.428096004595558</v>
+        <v>6.409117658226334</v>
       </c>
       <c r="E65">
-        <v>1.292121299730038E-10</v>
+        <v>1.463642110546665E-10</v>
       </c>
       <c r="F65">
-        <v>5.773882031411312E-08</v>
+        <v>6.227169905185825E-08</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -1996,19 +1996,19 @@
         <v>436.5933989727528</v>
       </c>
       <c r="B66">
-        <v>2.011466004289944</v>
+        <v>2.01145694734304</v>
       </c>
       <c r="C66">
-        <v>0.280238026317795</v>
+        <v>0.2807718096595023</v>
       </c>
       <c r="D66">
-        <v>7.177705433911759</v>
+        <v>7.164027434885201</v>
       </c>
       <c r="E66">
-        <v>7.089109083403936E-13</v>
+        <v>7.834071517821328E-13</v>
       </c>
       <c r="F66">
-        <v>4.142493627082923E-10</v>
+        <v>4.32063551747694E-10</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2018,22 +2018,22 @@
     </row>
     <row r="67">
       <c r="A67">
-        <v>61.76538459963529</v>
+        <v>61.7653845996353</v>
       </c>
       <c r="B67">
-        <v>3.274302909905705</v>
+        <v>3.274255757730848</v>
       </c>
       <c r="C67">
-        <v>0.6857924449132955</v>
+        <v>0.6879821837071619</v>
       </c>
       <c r="D67">
-        <v>4.774480871278298</v>
+        <v>4.759215914702419</v>
       </c>
       <c r="E67">
-        <v>1.801714067677236E-06</v>
+        <v>1.943464513004713E-06</v>
       </c>
       <c r="F67">
-        <v>0.0002793208350022474</v>
+        <v>0.0002953074496240121</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2043,22 +2043,22 @@
     </row>
     <row r="68">
       <c r="A68">
-        <v>57.71735554004748</v>
+        <v>57.71735554004749</v>
       </c>
       <c r="B68">
-        <v>2.048010142060397</v>
+        <v>2.047966150844558</v>
       </c>
       <c r="C68">
-        <v>0.5967655130650896</v>
+        <v>0.599503626509442</v>
       </c>
       <c r="D68">
-        <v>3.431850697171603</v>
+        <v>3.416103023043687</v>
       </c>
       <c r="E68">
-        <v>0.0005994774897067543</v>
+        <v>0.0006352420919114318</v>
       </c>
       <c r="F68">
-        <v>0.03212583695662986</v>
+        <v>0.03307479017710885</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2071,19 +2071,19 @@
         <v>100.5242003969598</v>
       </c>
       <c r="B69">
-        <v>2.842895775252215</v>
+        <v>2.842901360666739</v>
       </c>
       <c r="C69">
-        <v>0.4712991035053437</v>
+        <v>0.4731541279644154</v>
       </c>
       <c r="D69">
-        <v>6.032041550912862</v>
+        <v>6.008404434507113</v>
       </c>
       <c r="E69">
-        <v>1.619011339536443E-09</v>
+        <v>1.873579988537073E-09</v>
       </c>
       <c r="F69">
-        <v>5.590372563994814E-07</v>
+        <v>6.199884357623457E-07</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2093,22 +2093,22 @@
     </row>
     <row r="70">
       <c r="A70">
-        <v>56.59052948814021</v>
+        <v>56.59052948814022</v>
       </c>
       <c r="B70">
-        <v>2.716133500767082</v>
+        <v>2.716149872195403</v>
       </c>
       <c r="C70">
-        <v>0.5781593161421036</v>
+        <v>0.5808882614292609</v>
       </c>
       <c r="D70">
-        <v>4.697898010000229</v>
+        <v>4.675856016632846</v>
       </c>
       <c r="E70">
-        <v>2.628526220013182E-06</v>
+        <v>2.927299480518458E-06</v>
       </c>
       <c r="F70">
-        <v>0.0003953980085213888</v>
+        <v>0.0004191386208115419</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2118,22 +2118,22 @@
     </row>
     <row r="71">
       <c r="A71">
-        <v>89.07897202265092</v>
+        <v>89.07897202265094</v>
       </c>
       <c r="B71">
-        <v>2.993555477169429</v>
+        <v>2.993695574957922</v>
       </c>
       <c r="C71">
-        <v>0.5254601851194717</v>
+        <v>0.5273987362111608</v>
       </c>
       <c r="D71">
-        <v>5.697016752066185</v>
+        <v>5.676341958012014</v>
       </c>
       <c r="E71">
-        <v>1.219219520275281E-08</v>
+        <v>1.376055680960283E-08</v>
       </c>
       <c r="F71">
-        <v>3.430296698433766E-06</v>
+        <v>3.659079490210638E-06</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2143,22 +2143,22 @@
     </row>
     <row r="72">
       <c r="A72">
-        <v>19.70507673947992</v>
+        <v>19.70507673947993</v>
       </c>
       <c r="B72">
-        <v>4.198589431396207</v>
+        <v>4.198345177244172</v>
       </c>
       <c r="C72">
-        <v>1.199987298207481</v>
+        <v>1.204934120481741</v>
       </c>
       <c r="D72">
-        <v>3.498861561008172</v>
+        <v>3.484294374173458</v>
       </c>
       <c r="E72">
-        <v>0.0004672491135397023</v>
+        <v>0.000493436452368734</v>
       </c>
       <c r="F72">
-        <v>0.02648849172391305</v>
+        <v>0.02709765835198275</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2168,22 +2168,22 @@
     </row>
     <row r="73">
       <c r="A73">
-        <v>437.8637350102763</v>
+        <v>437.8637350102765</v>
       </c>
       <c r="B73">
-        <v>2.7836981338123</v>
+        <v>2.783698167883029</v>
       </c>
       <c r="C73">
-        <v>0.2565902071269341</v>
+        <v>0.257133873713125</v>
       </c>
       <c r="D73">
-        <v>10.84880894318471</v>
+        <v>10.82587108297019</v>
       </c>
       <c r="E73">
-        <v>2.020409135193527E-27</v>
+        <v>2.595988540773596E-27</v>
       </c>
       <c r="F73">
-        <v>6.139215198199052E-24</v>
+        <v>7.731373072131922E-24</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2196,19 +2196,19 @@
         <v>26.8642953318542</v>
       </c>
       <c r="B74">
-        <v>3.270906401018422</v>
+        <v>3.270852271783868</v>
       </c>
       <c r="C74">
-        <v>0.8981679921756552</v>
+        <v>0.9019981842748439</v>
       </c>
       <c r="D74">
-        <v>3.641753468741657</v>
+        <v>3.626229330398764</v>
       </c>
       <c r="E74">
-        <v>0.000270787330125504</v>
+        <v>0.0002875899676178106</v>
       </c>
       <c r="F74">
-        <v>0.01804417502893325</v>
+        <v>0.0186195748165079</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2218,22 +2218,22 @@
     </row>
     <row r="75">
       <c r="A75">
-        <v>28.79169656210055</v>
+        <v>28.79169656210056</v>
       </c>
       <c r="B75">
-        <v>3.184336075452104</v>
+        <v>3.184735341450573</v>
       </c>
       <c r="C75">
-        <v>0.9342754938646664</v>
+        <v>0.9380923612452516</v>
       </c>
       <c r="D75">
-        <v>3.408348069026167</v>
+        <v>3.394905952781729</v>
       </c>
       <c r="E75">
-        <v>0.0006535746915272155</v>
+        <v>0.0006865217878114609</v>
       </c>
       <c r="F75">
-        <v>0.0341228875889106</v>
+        <v>0.03483383060139323</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2246,19 +2246,19 @@
         <v>162.1724425170763</v>
       </c>
       <c r="B76">
-        <v>2.810996471287302</v>
+        <v>2.810981928942583</v>
       </c>
       <c r="C76">
-        <v>0.3903898839385322</v>
+        <v>0.3917715286668432</v>
       </c>
       <c r="D76">
-        <v>7.20048491761098</v>
+        <v>7.175054140631545</v>
       </c>
       <c r="E76">
-        <v>5.999879437500288E-13</v>
+        <v>7.227857698727868E-13</v>
       </c>
       <c r="F76">
-        <v>3.646246731757675E-10</v>
+        <v>4.139616499682949E-10</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2268,22 +2268,22 @@
     </row>
     <row r="77">
       <c r="A77">
-        <v>39.07070592499769</v>
+        <v>39.0707059249977</v>
       </c>
       <c r="B77">
-        <v>2.481254624897814</v>
+        <v>2.481299765734046</v>
       </c>
       <c r="C77">
-        <v>0.696306296688632</v>
+        <v>0.6996225942898994</v>
       </c>
       <c r="D77">
-        <v>3.563452803310437</v>
+        <v>3.546626118118022</v>
       </c>
       <c r="E77">
-        <v>0.0003660085269242992</v>
+        <v>0.0003901979256762031</v>
       </c>
       <c r="F77">
-        <v>0.0225132289455906</v>
+        <v>0.02352403769734551</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2293,22 +2293,22 @@
     </row>
     <row r="78">
       <c r="A78">
-        <v>48.73215432400341</v>
+        <v>48.73215432400342</v>
       </c>
       <c r="B78">
-        <v>2.514758719819366</v>
+        <v>2.514811997346071</v>
       </c>
       <c r="C78">
-        <v>0.6441494808344206</v>
+        <v>0.6470676677447004</v>
       </c>
       <c r="D78">
-        <v>3.903998675217109</v>
+        <v>3.886474510635396</v>
       </c>
       <c r="E78">
-        <v>9.461629854563536E-05</v>
+        <v>0.0001017106008720139</v>
       </c>
       <c r="F78">
-        <v>0.007770299588128853</v>
+        <v>0.008142863212823436</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2318,22 +2318,22 @@
     </row>
     <row r="79">
       <c r="A79">
-        <v>97.9639188564249</v>
+        <v>97.96391885642491</v>
       </c>
       <c r="B79">
-        <v>2.140488662302074</v>
+        <v>2.140338735895481</v>
       </c>
       <c r="C79">
-        <v>0.5001514236039933</v>
+        <v>0.5018839847214256</v>
       </c>
       <c r="D79">
-        <v>4.279681235091028</v>
+        <v>4.264608557062229</v>
       </c>
       <c r="E79">
-        <v>1.871611789351639E-05</v>
+        <v>2.002529649214339E-05</v>
       </c>
       <c r="F79">
-        <v>0.002122044620568616</v>
+        <v>0.002176618175653338</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2343,22 +2343,22 @@
     </row>
     <row r="80">
       <c r="A80">
-        <v>63.96406702799979</v>
+        <v>63.9640670279998</v>
       </c>
       <c r="B80">
-        <v>2.979864675063563</v>
+        <v>2.979722036402269</v>
       </c>
       <c r="C80">
-        <v>0.7128945594766342</v>
+        <v>0.7153900030225114</v>
       </c>
       <c r="D80">
-        <v>4.179951488550013</v>
+        <v>4.165171478232839</v>
       </c>
       <c r="E80">
-        <v>2.915712893029858E-05</v>
+        <v>3.111186314801227E-05</v>
       </c>
       <c r="F80">
-        <v>0.003034138766013878</v>
+        <v>0.003130315906331423</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -2371,19 +2371,19 @@
         <v>38.6695722759781</v>
       </c>
       <c r="B81">
-        <v>3.146727447924272</v>
+        <v>3.146787501214695</v>
       </c>
       <c r="C81">
-        <v>0.7480759624029291</v>
+        <v>0.7512811706522413</v>
       </c>
       <c r="D81">
-        <v>4.206427697284277</v>
+        <v>4.188561651934843</v>
       </c>
       <c r="E81">
-        <v>2.594390338009981E-05</v>
+        <v>2.807280499712349E-05</v>
       </c>
       <c r="F81">
-        <v>0.002775814958125749</v>
+        <v>0.002903000966751152</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -2396,19 +2396,19 @@
         <v>984.0864592420047</v>
       </c>
       <c r="B82">
-        <v>2.79831433320376</v>
+        <v>2.7983123523396</v>
       </c>
       <c r="C82">
-        <v>0.2405536117756244</v>
+        <v>0.2406430783459298</v>
       </c>
       <c r="D82">
-        <v>11.63280947040561</v>
+        <v>11.62847637910019</v>
       </c>
       <c r="E82">
-        <v>2.807041153193953E-31</v>
+        <v>2.95321627458508E-31</v>
       </c>
       <c r="F82">
-        <v>1.421579208015857E-27</v>
+        <v>1.761113774623724E-27</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -2418,22 +2418,22 @@
     </row>
     <row r="83">
       <c r="A83">
-        <v>8044.623318304551</v>
+        <v>8044.623318304553</v>
       </c>
       <c r="B83">
-        <v>3.803837602428057</v>
+        <v>3.803837602428058</v>
       </c>
       <c r="C83">
-        <v>0.6958076176234756</v>
+        <v>0.6958076176234761</v>
       </c>
       <c r="D83">
-        <v>5.466794996323881</v>
+        <v>5.46679499632388</v>
       </c>
       <c r="E83">
-        <v>4.582455082277287E-08</v>
+        <v>4.582455082277334E-08</v>
       </c>
       <c r="F83">
-        <v>1.071096001000597E-05</v>
+        <v>1.066208416096747E-05</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -2446,19 +2446,19 @@
         <v>18.8604777773755</v>
       </c>
       <c r="B84">
-        <v>4.316308835005844</v>
+        <v>4.316728877312132</v>
       </c>
       <c r="C84">
-        <v>1.191287254238407</v>
+        <v>1.195575320016166</v>
       </c>
       <c r="D84">
-        <v>3.623230937499849</v>
+        <v>3.610587141639695</v>
       </c>
       <c r="E84">
-        <v>0.0002909458362586179</v>
+        <v>0.0003055046352475176</v>
       </c>
       <c r="F84">
-        <v>0.01894303367283356</v>
+        <v>0.01935859371689695</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -2468,22 +2468,22 @@
     </row>
     <row r="85">
       <c r="A85">
-        <v>58.57957461251223</v>
+        <v>58.57957461251224</v>
       </c>
       <c r="B85">
-        <v>2.148484241595848</v>
+        <v>2.148473725606877</v>
       </c>
       <c r="C85">
-        <v>0.5715003547578449</v>
+        <v>0.5741861216672971</v>
       </c>
       <c r="D85">
-        <v>3.759375166978154</v>
+        <v>3.741772300884304</v>
       </c>
       <c r="E85">
-        <v>0.0001703382439854025</v>
+        <v>0.0001827270421430533</v>
       </c>
       <c r="F85">
-        <v>0.01238253081756086</v>
+        <v>0.01292615530682281</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -2496,19 +2496,19 @@
         <v>1183.583600457755</v>
       </c>
       <c r="B86">
-        <v>2.011066174055907</v>
+        <v>2.011066018117109</v>
       </c>
       <c r="C86">
-        <v>0.2617085728030236</v>
+        <v>0.2617233196375298</v>
       </c>
       <c r="D86">
-        <v>7.684372554236302</v>
+        <v>7.68393898144922</v>
       </c>
       <c r="E86">
-        <v>1.537486441478127E-14</v>
+        <v>1.542701654212733E-14</v>
       </c>
       <c r="F86">
-        <v>1.557268767025146E-11</v>
+        <v>1.531491355525454E-11</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -2521,19 +2521,19 @@
         <v>126.8808120062238</v>
       </c>
       <c r="B87">
-        <v>2.334769400070957</v>
+        <v>2.334789948227279</v>
       </c>
       <c r="C87">
-        <v>0.4264789829345318</v>
+        <v>0.4281285166326855</v>
       </c>
       <c r="D87">
-        <v>5.474523935519148</v>
+        <v>5.453479171606832</v>
       </c>
       <c r="E87">
-        <v>4.386893463035759E-08</v>
+        <v>4.93937338759843E-08</v>
       </c>
       <c r="F87">
-        <v>1.041407380998473E-05</v>
+        <v>1.111355967997097E-05</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -2543,22 +2543,22 @@
     </row>
     <row r="88">
       <c r="A88">
-        <v>25.3787963033892</v>
+        <v>25.37879630338922</v>
       </c>
       <c r="B88">
-        <v>4.67428594904738</v>
+        <v>4.674423769808343</v>
       </c>
       <c r="C88">
-        <v>1.099494102252187</v>
+        <v>1.102891341230583</v>
       </c>
       <c r="D88">
-        <v>4.251306068375121</v>
+        <v>4.238335722712918</v>
       </c>
       <c r="E88">
-        <v>2.125274928814826E-05</v>
+        <v>2.251828642509177E-05</v>
       </c>
       <c r="F88">
-        <v>0.002339804492281424</v>
+        <v>0.002395141451114583</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -2568,22 +2568,22 @@
     </row>
     <row r="89">
       <c r="A89">
-        <v>31.01640839913327</v>
+        <v>31.01640839913328</v>
       </c>
       <c r="B89">
-        <v>8.410269432062092</v>
+        <v>8.410266588927191</v>
       </c>
       <c r="C89">
-        <v>1.621316157403189</v>
+        <v>1.623453317084379</v>
       </c>
       <c r="D89">
-        <v>5.187309947945351</v>
+        <v>5.180479475708919</v>
       </c>
       <c r="E89">
-        <v>2.133534761038464E-07</v>
+        <v>2.213162794871334E-07</v>
       </c>
       <c r="F89">
-        <v>4.321972483260984E-05</v>
+        <v>4.394160957123872E-05</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -2596,19 +2596,19 @@
         <v>66.77461528826194</v>
       </c>
       <c r="B90">
-        <v>2.580244810839935</v>
+        <v>2.580243550670374</v>
       </c>
       <c r="C90">
-        <v>0.6411698075022149</v>
+        <v>0.6434815347993947</v>
       </c>
       <c r="D90">
-        <v>4.024276846240958</v>
+        <v>4.009817548960072</v>
       </c>
       <c r="E90">
-        <v>5.71506558248007E-05</v>
+        <v>6.07656827572216E-05</v>
       </c>
       <c r="F90">
-        <v>0.005326931987399982</v>
+        <v>0.005450974589986667</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -2618,22 +2618,22 @@
     </row>
     <row r="91">
       <c r="A91">
-        <v>83.79989328536288</v>
+        <v>83.79989328536291</v>
       </c>
       <c r="B91">
-        <v>2.519716224273302</v>
+        <v>2.519737180963809</v>
       </c>
       <c r="C91">
-        <v>0.5014220254289801</v>
+        <v>0.5035303097750842</v>
       </c>
       <c r="D91">
-        <v>5.02514069284774</v>
+        <v>5.004142018956753</v>
       </c>
       <c r="E91">
-        <v>5.030635969949415E-07</v>
+        <v>5.611137949231535E-07</v>
       </c>
       <c r="F91">
-        <v>9.208488227884514E-05</v>
+        <v>9.83005355317727E-05</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -2646,19 +2646,19 @@
         <v>100.850485058239</v>
       </c>
       <c r="B92">
-        <v>3.208081400977774</v>
+        <v>3.208089043665391</v>
       </c>
       <c r="C92">
-        <v>0.4639236980965927</v>
+        <v>0.4657875925360346</v>
       </c>
       <c r="D92">
-        <v>6.915105682550895</v>
+        <v>6.887450621427201</v>
       </c>
       <c r="E92">
-        <v>4.675147099287798E-12</v>
+        <v>5.680107909417087E-12</v>
       </c>
       <c r="F92">
-        <v>2.449293444119983E-09</v>
+        <v>2.819416229304328E-09</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -2668,22 +2668,22 @@
     </row>
     <row r="93">
       <c r="A93">
-        <v>77.46595532121127</v>
+        <v>77.46595532121128</v>
       </c>
       <c r="B93">
-        <v>2.417700667253796</v>
+        <v>2.417302852292355</v>
       </c>
       <c r="C93">
-        <v>0.5865658973785016</v>
+        <v>0.5887768799395694</v>
       </c>
       <c r="D93">
-        <v>4.121788665278801</v>
+        <v>4.105634807773805</v>
       </c>
       <c r="E93">
-        <v>3.759420082291425E-05</v>
+        <v>4.032060555087933E-05</v>
       </c>
       <c r="F93">
-        <v>0.003757688770411423</v>
+        <v>0.003898793099078858</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -2696,19 +2696,19 @@
         <v>17.81361178574583</v>
       </c>
       <c r="B94">
-        <v>4.394674800441678</v>
+        <v>4.394791313600159</v>
       </c>
       <c r="C94">
-        <v>1.127228057070114</v>
+        <v>1.131866554414821</v>
       </c>
       <c r="D94">
-        <v>3.898656330347469</v>
+        <v>3.882782202953494</v>
       </c>
       <c r="E94">
-        <v>9.672794375931352E-05</v>
+        <v>0.0001032680586239047</v>
       </c>
       <c r="F94">
-        <v>0.007858757484145724</v>
+        <v>0.008179599260471094</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -2721,19 +2721,19 @@
         <v>46.51710651503814</v>
       </c>
       <c r="B95">
-        <v>2.653699355236432</v>
+        <v>2.653720549537287</v>
       </c>
       <c r="C95">
-        <v>0.6530063442634835</v>
+        <v>0.6559718333606618</v>
       </c>
       <c r="D95">
-        <v>4.063818642113656</v>
+        <v>4.045479416306336</v>
       </c>
       <c r="E95">
-        <v>4.827634119767258E-05</v>
+        <v>5.221615381759526E-05</v>
       </c>
       <c r="F95">
-        <v>0.004612971395070688</v>
+        <v>0.004829507742222429</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>

</xml_diff>